<commit_message>
scan: seg0 2026-08-31 18:04 CST
</commit_message>
<xml_diff>
--- a/output/full_scan/batch_seq1_2026-08-31.xlsx
+++ b/output/full_scan/batch_seq1_2026-08-31.xlsx
@@ -5626,7 +5626,7 @@
         <v/>
       </c>
       <c r="D98" s="2" t="n">
-        <v>235.6610551174354</v>
+        <v>235.6610551174353</v>
       </c>
       <c r="E98" s="2" t="n">
         <v>16.3</v>
@@ -6368,7 +6368,7 @@
         <v/>
       </c>
       <c r="D112" s="2" t="n">
-        <v>202.2903562681362</v>
+        <v>202.2903562681361</v>
       </c>
       <c r="E112" s="2" t="n">
         <v>17.3</v>

</xml_diff>